<commit_message>
Updating Recent Changes - 19-09-2026
</commit_message>
<xml_diff>
--- a/Data Engineering Plan.xlsx
+++ b/Data Engineering Plan.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_2843813722E71A4784B04B253E8DBFD7F01055EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2B85F23-14A2-4960-BD30-8CFA21D39C9C}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChandrG\DE Track\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EF7368-0CEE-454E-BAFE-D25E3191CEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Engineering Plan" sheetId="1" r:id="rId1"/>
@@ -35,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="206">
   <si>
     <t>Serial No.</t>
   </si>
@@ -644,13 +649,22 @@
   </si>
   <si>
     <t>DP-700, Databricks Data Engineer Associate, Google Professional Data Engineer (optional in 6 months; continue if needed)</t>
+  </si>
+  <si>
+    <t>In-Progress</t>
+  </si>
+  <si>
+    <t>Have completed File Handling module and also added few extra course links</t>
+  </si>
+  <si>
+    <t>I think we need to break this section into sub-groups, since post learning the "File Handling" conncepts other part of course track like "API ingestion" I am finding it a bit difficult to learn the concept from the given links.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -737,7 +751,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{C4B67E71-DB29-44CB-BC87-73CB116A2270}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1035,7 +1051,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
@@ -1043,7 +1059,7 @@
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="70" customWidth="1"/>
-    <col min="8" max="8" width="45" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" customWidth="1"/>
     <col min="9" max="10" width="50" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
@@ -1053,7 +1069,7 @@
     <col min="16" max="17" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1106,7 +1122,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="30.75">
+    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1143,11 +1159,13 @@
       <c r="N2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="2"/>
+      <c r="O2" s="2">
+        <v>100</v>
+      </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" spans="1:17" ht="30.75">
+    <row r="3" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1184,11 +1202,13 @@
       <c r="N3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="2"/>
+      <c r="O3" s="2">
+        <v>100</v>
+      </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
-    <row r="4" spans="1:17" ht="57.75" customHeight="1">
+    <row r="4" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1221,13 +1241,19 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-    </row>
-    <row r="5" spans="1:17">
+        <v>203</v>
+      </c>
+      <c r="O4" s="2">
+        <v>25</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1266,7 +1292,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1305,7 +1331,7 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1344,7 +1370,7 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1383,7 +1409,7 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="1:17" ht="30.75">
+    <row r="9" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1422,7 +1448,7 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1461,7 +1487,7 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1500,7 +1526,7 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1539,7 +1565,7 @@
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1578,7 +1604,7 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1617,7 +1643,7 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1656,7 +1682,7 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1695,7 +1721,7 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1734,7 +1760,7 @@
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1773,7 +1799,7 @@
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1812,7 +1838,7 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1851,7 +1877,7 @@
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1890,7 +1916,7 @@
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1929,7 +1955,7 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1968,7 +1994,7 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2007,7 +2033,7 @@
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2060,13 +2086,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>187</v>
       </c>
@@ -2074,7 +2100,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>189</v>
       </c>
@@ -2082,7 +2108,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>190</v>
       </c>
@@ -2090,7 +2116,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>191</v>
       </c>
@@ -2098,7 +2124,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>193</v>
       </c>
@@ -2106,7 +2132,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>195</v>
       </c>
@@ -2114,7 +2140,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>197</v>
       </c>
@@ -2122,7 +2148,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>199</v>
       </c>
@@ -2130,7 +2156,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="43.5" customHeight="1">
+    <row r="9" spans="1:2" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>201</v>
       </c>

</xml_diff>